<commit_message>
word onset + features
</commit_message>
<xml_diff>
--- a/data/phoneme_onset_D/St01_D.xlsx
+++ b/data/phoneme_onset_D/St01_D.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveunibo-my.sharepoint.com/personal/francesca_schiavon10_studio_unibo_it/Documents/Desktop/IMT/TESI/linguistic_pipeline_EEG/data/phoneme_onset_1115/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveunibo-my.sharepoint.com/personal/francesca_schiavon10_studio_unibo_it/Documents/Desktop/IMT/TESI/linguistic_pipeline_EEG/data/phoneme_onset_D/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_3151B3A2D3F0523B4FF83E11595ED87656DD844B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E813D175-8033-45FD-9EEA-89C22BA2609B}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_3151B3A2D3F0523B4FF83E11595ED87656DD844B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0397BAA7-3BDE-43C8-A7FC-80789844940F}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="12090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6144" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6145" uniqueCount="580">
   <si>
     <t>BEGIN</t>
   </si>
@@ -1757,6 +1757,9 @@
   </si>
   <si>
     <t>m o n d o</t>
+  </si>
+  <si>
+    <t>=</t>
   </si>
 </sst>
 </file>
@@ -1839,10 +1842,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2296,6 +2295,9 @@
       <c r="G7" t="s">
         <v>20</v>
       </c>
+      <c r="M7" t="s">
+        <v>579</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8">

</xml_diff>